<commit_message>
Dashboard update 2026-09-01 22:40
</commit_message>
<xml_diff>
--- a/excel/Revolut Brokerage Rima.xlsx
+++ b/excel/Revolut Brokerage Rima.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.08.08\Revolut\Brokerage Account Rima\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69be8bcaca992739/Dokumentai/portfolio-analytics/portfolio-dashboard-clean/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EE1FC9-214D-466E-AEDD-AC0AB94F2565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C1EE1FC9-214D-466E-AEDD-AC0AB94F2565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{423C2149-F0E0-425C-A1BC-50329235457A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apžvalga" sheetId="81" r:id="rId1"/>
@@ -646,24 +646,6 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -689,6 +671,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1893,18 +1893,54 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
+      <c r="A10" s="36">
+        <f>'2026.08'!$Q$2</f>
+        <v>2026.08</v>
+      </c>
+      <c r="B10" s="4">
+        <f>B9+'2026.08'!$Q$5</f>
+        <v>800</v>
+      </c>
+      <c r="C10" s="4">
+        <f>'2026.08'!$R$5</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="4">
+        <f>D9+'2026.08'!$S$5-K10-L10</f>
+        <v>800</v>
+      </c>
+      <c r="E10" s="4">
+        <f>'2026.08'!$X$5</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <f>WEBN!H12</f>
+        <v>860.34665192519992</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" ref="G10" si="6">SUM(F10:F10)+E10</f>
+        <v>860.34665192519992</v>
+      </c>
+      <c r="H10" s="4">
+        <f t="shared" ref="H10" si="7">G10-B10</f>
+        <v>60.346651925199922</v>
+      </c>
+      <c r="I10" s="21">
+        <f t="shared" ref="I10" si="8">H10/B10</f>
+        <v>7.5433314906499904E-2</v>
+      </c>
+      <c r="J10" s="4">
+        <f>'2026.08'!$W$5</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="4">
+        <f>'2026.08'!$U$5</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="4">
+        <f>'2026.08'!$V$5</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
@@ -2021,6 +2057,7 @@
     <hyperlink ref="F2" location="WEBN!A1" display="WEBN!A1" xr:uid="{499756ED-B1F9-4D05-897B-F69DF5557EF9}"/>
     <hyperlink ref="A8" location="'2026.06'!A1" display="'2026.06'!A1" xr:uid="{EDD493B5-6E5A-4B6F-9C2F-600CF21AFF32}"/>
     <hyperlink ref="A9" location="'2026.07'!A1" display="'2026.07'!A1" xr:uid="{0EA64D34-DE59-4B69-AFFB-31BBE94C6E84}"/>
+    <hyperlink ref="A10" location="'2026.08'!A1" display="'2026.08'!A1" xr:uid="{EBA7FF03-B603-4FA0-A3D1-936DE1CCCC75}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2044,34 +2081,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.08</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -2126,23 +2163,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -2153,14 +2190,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -2187,7 +2224,7 @@
       <c r="F14" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="56" t="s">
         <v>32</v>
       </c>
@@ -2232,7 +2269,7 @@
       <c r="F15" s="13">
         <v>7.7519379800000001</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -2250,7 +2287,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -2267,7 +2304,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -2284,7 +2321,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -2318,7 +2355,7 @@
         <f>SUM(F15:F18)</f>
         <v>7.7519379800000001</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="56" t="s">
         <v>2</v>
       </c>
@@ -2363,11 +2400,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A12:O12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="G13:G19"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="N13:O13"/>
     <mergeCell ref="Q2:X2"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="R3:R4"/>
@@ -2376,6 +2408,11 @@
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="X3:X4"/>
+    <mergeCell ref="A12:O12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:G19"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="N13:O13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A12:O12" location="WEBN!A1" display="WEBN Amundi Prime ACWI Acc UCITS ETF " xr:uid="{3CE52383-29C5-4497-90B8-DA81B24EC7D1}"/>
@@ -2406,34 +2443,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.07</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -2488,23 +2525,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -2515,14 +2552,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -2549,7 +2586,7 @@
       <c r="F14" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="50" t="s">
         <v>32</v>
       </c>
@@ -2594,7 +2631,7 @@
       <c r="F15" s="13">
         <v>7.8382191499999996</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -2612,7 +2649,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -2629,7 +2666,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -2646,7 +2683,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -2680,7 +2717,7 @@
         <f>SUM(F15:F18)</f>
         <v>7.8382191499999996</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="50" t="s">
         <v>2</v>
       </c>
@@ -2725,11 +2762,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A12:O12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="G13:G19"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="N13:O13"/>
     <mergeCell ref="Q2:X2"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="R3:R4"/>
@@ -2738,6 +2770,11 @@
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="X3:X4"/>
+    <mergeCell ref="A12:O12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:G19"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="N13:O13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A12:O12" location="WEBN!A1" display="WEBN Amundi Prime ACWI Acc UCITS ETF " xr:uid="{DF2B807C-B133-4C46-9D1B-D6B7BEF50215}"/>
@@ -2768,34 +2805,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.06</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -2850,23 +2887,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -2877,14 +2914,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -2911,7 +2948,7 @@
       <c r="F14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="3" t="s">
         <v>32</v>
       </c>
@@ -2956,7 +2993,7 @@
       <c r="F15" s="13">
         <v>8.05542129</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -2974,7 +3011,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -2991,7 +3028,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3008,7 +3045,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -3042,7 +3079,7 @@
         <f>SUM(F15:F18)</f>
         <v>8.05542129</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="3" t="s">
         <v>2</v>
       </c>
@@ -3087,6 +3124,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:G19"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="X3:X4"/>
@@ -3095,11 +3137,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="G13:G19"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="Q3:Q4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A12:O12" location="WEBN!A1" display="WEBN Amundi Prime ACWI Acc UCITS ETF " xr:uid="{52D9614F-EF79-46CC-8F5E-FBD95649CF20}"/>
@@ -3130,34 +3167,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.05</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -3212,23 +3249,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -3239,14 +3276,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -3273,7 +3310,7 @@
       <c r="F14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="3" t="s">
         <v>32</v>
       </c>
@@ -3318,7 +3355,7 @@
       <c r="F15" s="13">
         <v>8.1859855899999996</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -3336,7 +3373,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -3353,7 +3390,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3370,7 +3407,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -3404,7 +3441,7 @@
         <f>SUM(F15:F18)</f>
         <v>8.1859855899999996</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="3" t="s">
         <v>2</v>
       </c>
@@ -3449,6 +3486,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:G19"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="X3:X4"/>
@@ -3457,11 +3499,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="G13:G19"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="Q3:Q4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A12:O12" location="WEBN!A1" display="WEBN Amundi Prime ACWI Acc UCITS ETF " xr:uid="{3C02C9E5-EA02-4BDC-91AE-416C94F85838}"/>
@@ -3492,34 +3529,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.04</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -3574,23 +3611,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -3601,14 +3638,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -3635,7 +3672,7 @@
       <c r="F14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="3" t="s">
         <v>32</v>
       </c>
@@ -3680,7 +3717,7 @@
       <c r="F15" s="13">
         <v>8.6236633299999994</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -3698,7 +3735,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -3715,7 +3752,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3732,7 +3769,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -3766,7 +3803,7 @@
         <f>SUM(F15:F18)</f>
         <v>8.6236633299999994</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="3" t="s">
         <v>2</v>
       </c>
@@ -3811,6 +3848,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:G19"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="X3:X4"/>
@@ -3819,11 +3861,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="G13:G19"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="Q3:Q4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A12:O12" location="WEBN!A1" display="WEBN Amundi Prime ACWI Acc UCITS ETF " xr:uid="{5E453430-7CF8-4213-8F80-26238D76E7AB}"/>
@@ -3854,34 +3891,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.03</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -3936,23 +3973,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -3963,14 +4000,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -3997,7 +4034,7 @@
       <c r="F14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="3" t="s">
         <v>32</v>
       </c>
@@ -4042,7 +4079,7 @@
       <c r="F15" s="13">
         <v>9.0073860499999991</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -4060,7 +4097,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -4077,7 +4114,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -4094,7 +4131,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -4128,7 +4165,7 @@
         <f>SUM(F15:F18)</f>
         <v>9.0073860499999991</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="3" t="s">
         <v>2</v>
       </c>
@@ -4173,6 +4210,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:G19"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="X3:X4"/>
@@ -4181,11 +4223,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="G13:G19"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="Q3:Q4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A12:O12" location="WEBN!A1" display="WEBN Amundi Prime ACWI Acc UCITS ETF " xr:uid="{04427A72-C2D7-400B-ACC4-6F6AA44B6641}"/>
@@ -4216,34 +4253,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.02</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -4298,23 +4335,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -4325,14 +4362,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -4359,7 +4396,7 @@
       <c r="F14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="3" t="s">
         <v>32</v>
       </c>
@@ -4404,7 +4441,7 @@
       <c r="F15" s="13">
         <v>8.7032201899999997</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -4422,7 +4459,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -4439,7 +4476,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -4456,7 +4493,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -4490,7 +4527,7 @@
         <f>SUM(F15:F18)</f>
         <v>8.7032201899999997</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="3" t="s">
         <v>2</v>
       </c>
@@ -4535,6 +4572,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:G19"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="X3:X4"/>
@@ -4543,11 +4585,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="G13:G19"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="Q3:Q4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A12:O12" location="WEBN!A1" display="WEBN Amundi Prime ACWI Acc UCITS ETF " xr:uid="{BF7DD392-2323-41A9-A80E-2E9F0505699A}"/>
@@ -4578,34 +4615,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q2" s="71">
+      <c r="Q2" s="80">
         <v>2026.01</v>
       </c>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="82"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="74" t="s">
+      <c r="R3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="74" t="s">
+      <c r="S3" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="74" t="s">
+      <c r="T3" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="75" t="s">
+      <c r="U3" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="76"/>
+      <c r="V3" s="85"/>
       <c r="W3" s="68" t="s">
         <v>39</v>
       </c>
@@ -4660,23 +4697,23 @@
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="79"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="80"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="73"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="74"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
@@ -4687,14 +4724,14 @@
       <c r="D13" s="66"/>
       <c r="E13" s="66"/>
       <c r="F13" s="63"/>
-      <c r="G13" s="81"/>
-      <c r="H13" s="84" t="s">
+      <c r="G13" s="75"/>
+      <c r="H13" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
       <c r="M13" s="30"/>
       <c r="N13" s="62" t="s">
         <v>39</v>
@@ -4721,7 +4758,7 @@
       <c r="F14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="82"/>
+      <c r="G14" s="76"/>
       <c r="H14" s="3" t="s">
         <v>32</v>
       </c>
@@ -4766,7 +4803,7 @@
       <c r="F15" s="13">
         <v>8.7351502399999994</v>
       </c>
-      <c r="G15" s="82"/>
+      <c r="G15" s="76"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="4"/>
@@ -4784,7 +4821,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
-      <c r="G16" s="82"/>
+      <c r="G16" s="76"/>
       <c r="H16" s="5"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -4801,7 +4838,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="82"/>
+      <c r="G17" s="76"/>
       <c r="H17" s="5"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -4818,7 +4855,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="82"/>
+      <c r="G18" s="76"/>
       <c r="H18" s="5"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -4852,7 +4889,7 @@
         <f>SUM(F15:F18)</f>
         <v>8.7351502399999994</v>
       </c>
-      <c r="G19" s="83"/>
+      <c r="G19" s="77"/>
       <c r="H19" s="3" t="s">
         <v>2</v>
       </c>
@@ -7266,6 +7303,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
@@ -7273,12 +7316,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="K3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7707,6 +7744,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
@@ -7714,12 +7757,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="K3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8483,6 +8520,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="K3:L3"/>
@@ -8491,11 +8533,6 @@
     <mergeCell ref="P3:P4"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="R3:R4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="S3:S4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -9581,24 +9618,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="S3:U3"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="AC3:AC4"/>
     <mergeCell ref="AD3:AD4"/>
     <mergeCell ref="AE3:AE4"/>
     <mergeCell ref="X3:X4"/>
     <mergeCell ref="AF3:AG3"/>
     <mergeCell ref="Y3:Y4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="V3:W3"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="R3:R4"/>
-    <mergeCell ref="S3:U3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A5" location="'2026.01'!A1" display="'2026.01'!A1" xr:uid="{BAF6215B-37D5-4AB2-9B9C-F1057A1F97E5}"/>

</xml_diff>